<commit_message>
feat(vision): add on-demand water level predictor, label studio active learning loop, and clean raw frames
</commit_message>
<xml_diff>
--- a/workers/vision/water_levels.xlsx
+++ b/workers/vision/water_levels.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -549,6 +549,42 @@
         <v>0.6</v>
       </c>
     </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:05:03</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>10.19</v>
+      </c>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:05:04</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:05:05</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="7" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>